<commit_message>
deskos: upgrade all 3 customer strata to 10 permanent free instruments (30 total) across xlsx, guides & Whop zip packs
</commit_message>
<xml_diff>
--- a/deskos/xlsx/DeskOS_Founder_And_Seller_CRM_Command_OS.xlsx
+++ b/deskos/xlsx/DeskOS_Founder_And_Seller_CRM_Command_OS.xlsx
@@ -616,7 +616,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://stpi-leads.stpi-cloud.workers.dev/deskos/deskos-co-andina-customs-ip-counse-7351bf75</t>
+          <t>https://stpi-deskos.stpi-cloud.workers.dev/os/deskos-co-andina-customs-ip-counse-7351bf75</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://stpi-leads.stpi-cloud.workers.dev/deskos/deskos-bw-okavango-sovereign-exped-910d455c</t>
+          <t>https://stpi-deskos.stpi-cloud.workers.dev/os/deskos-bw-okavango-sovereign-exped-910d455c</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://stpi-leads.stpi-cloud.workers.dev/deskos/deskos-jo-al-masar-infrastructure--dbb9d86a</t>
+          <t>https://stpi-deskos.stpi-cloud.workers.dev/os/deskos-jo-al-masar-infrastructure--dbb9d86a</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://stpi-leads.stpi-cloud.workers.dev/deskos/deskos-vn-mekong-delta-freight-ip--af34e3ee</t>
+          <t>https://stpi-deskos.stpi-cloud.workers.dev/os/deskos-vn-mekong-delta-freight-ip--af34e3ee</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://stpi-leads.stpi-cloud.workers.dev/deskos/deskos-ro-danube-aegean-engineerin-c36521a7</t>
+          <t>https://stpi-deskos.stpi-cloud.workers.dev/os/deskos-ro-danube-aegean-engineerin-c36521a7</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://stpi-leads.stpi-cloud.workers.dev/deskos/deskos-mu-coral-harbour-luxury-dmc-cf456208</t>
+          <t>https://stpi-deskos.stpi-cloud.workers.dev/os/deskos-mu-coral-harbour-luxury-dmc-cf456208</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">

</xml_diff>